<commit_message>
Integrate validated graphs with paginated evidence panel and year corpus counts
</commit_message>
<xml_diff>
--- a/validation_1990_age32/edge_validation.xlsx
+++ b/validation_1990_age32/edge_validation.xlsx
@@ -151,17 +151,19 @@
       </c>
       <c r="G2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The new family study supports familial ADD liability across relatives but supplies no adult age-specific genetic effect; the adult review describes persistence without establishing a genetic cause.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Obtain adult genetic-liability evidence with the relevant phenotype and age scope.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2387786: These results confirm and extend previous findings indicating important family-genetic risk factors in ADD.
+Location: Family-genetic and psychosocial risk factors in DSM-III attention deficit disorder - PubMed.html; English abstract (#eng-abstract)
+Relevance: Blinded family study supports familial liability; shared environment is not fully separated and strong genetic causation or an exact-age effect is not established.</t>
         </is>
       </c>
     </row>
@@ -292,7 +294,7 @@
       </c>
       <c r="G5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr" s="0">
@@ -339,7 +341,7 @@
       </c>
       <c r="G6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr" s="0">
@@ -386,7 +388,7 @@
       </c>
       <c r="G7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr" s="0">
@@ -433,7 +435,7 @@
       </c>
       <c r="G8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr" s="0">
@@ -480,7 +482,7 @@
       </c>
       <c r="G9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr" s="0">
@@ -574,7 +576,7 @@
       </c>
       <c r="G11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="0">
@@ -621,7 +623,7 @@
       </c>
       <c r="G12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H12" t="inlineStr" s="0">
@@ -668,7 +670,7 @@
       </c>
       <c r="G13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="0">
@@ -715,7 +717,7 @@
       </c>
       <c r="G14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr" s="0">
@@ -762,7 +764,7 @@
       </c>
       <c r="G15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H15" t="inlineStr" s="0">
@@ -809,7 +811,7 @@
       </c>
       <c r="G16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr" s="0">
@@ -856,7 +858,7 @@
       </c>
       <c r="G17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H17" t="inlineStr" s="0">
@@ -903,7 +905,7 @@
       </c>
       <c r="G18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H18" t="inlineStr" s="0">
@@ -950,7 +952,7 @@
       </c>
       <c r="G19" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H19" t="inlineStr" s="0">
@@ -997,7 +999,7 @@
       </c>
       <c r="G20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H20" t="inlineStr" s="0">
@@ -1044,7 +1046,7 @@
       </c>
       <c r="G21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H21" t="inlineStr" s="0">
@@ -1091,7 +1093,7 @@
       </c>
       <c r="G22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H22" t="inlineStr" s="0">
@@ -1138,7 +1140,7 @@
       </c>
       <c r="G23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H23" t="inlineStr" s="0">
@@ -1185,7 +1187,7 @@
       </c>
       <c r="G24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H24" t="inlineStr" s="0">
@@ -1232,7 +1234,7 @@
       </c>
       <c r="G25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr" s="0">
@@ -1326,7 +1328,7 @@
       </c>
       <c r="G27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr" s="0">
@@ -1373,7 +1375,7 @@
       </c>
       <c r="G28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H28" t="inlineStr" s="0">
@@ -1420,7 +1422,7 @@
       </c>
       <c r="G29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr" s="0">
@@ -1462,22 +1464,24 @@
       </c>
       <c r="F30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">insufficient_evidence</t>
+          <t xml:space="preserve">partially_supported</t>
         </is>
       </c>
       <c r="G30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The adult review states that other diagnostic labels can mask ADHD. This provides clinical support for obscured recognition, but labels are not necessarily true comorbid conditions and the abstract does not quantify diagnostic errors at age 32.</t>
         </is>
       </c>
       <c r="H30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Restrict to diagnostic masking as a clinical hypothesis; distinguish true comorbidity from prior mislabeling.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Detection of the disorder later in life may be made more difficult when it is masked by other diagnostic labels.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult review and clinical experience support diagnostic masking; other labels may be mislabels rather than true comorbidity, and no age-32 or error-rate estimate is given.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1565,7 @@
       </c>
       <c r="G32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H32" t="inlineStr" s="0">
@@ -1608,7 +1612,7 @@
       </c>
       <c r="G33" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr" s="0">
@@ -1655,7 +1659,7 @@
       </c>
       <c r="G34" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H34" t="inlineStr" s="0">
@@ -1702,7 +1706,7 @@
       </c>
       <c r="G35" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr" s="0">
@@ -1749,17 +1753,19 @@
       </c>
       <c r="G36" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The new adult review mentions combined psychotherapy and medical management without naming medication or reporting drug-specific outcomes. Pediatric trials cannot supply an adult treatment-effect or medication-uptake estimate.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Obtain adult medication-specific evidence; do not interpret unspecified medical management as a drug trial.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -1791,22 +1797,24 @@
       </c>
       <c r="F37" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">insufficient_evidence</t>
+          <t xml:space="preserve">partially_supported</t>
         </is>
       </c>
       <c r="G37" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The adult review describes identification followed by psychotherapy and medical management. This supports a broader psychological-care pathway compatible with coping support; it does not identify a behavioral modality or estimate access at age 32.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Label the supporting evidence as psychotherapy broadly; obtain evidence specific to behavioral/coping treatment and adult referral rates.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1851,7 @@
       </c>
       <c r="G38" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr" s="0">
@@ -1890,7 +1898,7 @@
       </c>
       <c r="G39" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr" s="0">
@@ -1937,7 +1945,7 @@
       </c>
       <c r="G40" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr" s="0">
@@ -1984,7 +1992,7 @@
       </c>
       <c r="G41" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr" s="0">
@@ -2031,7 +2039,7 @@
       </c>
       <c r="G42" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H42" t="inlineStr" s="0">
@@ -2078,7 +2086,7 @@
       </c>
       <c r="G43" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr" s="0">
@@ -2125,17 +2133,19 @@
       </c>
       <c r="G44" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The adult review does not specify behavioral therapy or isolate its effect on functional impairment. Preschool parent training and child medication studies do not establish this adult claim.</t>
         </is>
       </c>
       <c r="H44" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Obtain adult behavioral-treatment evidence with separately measured functional outcomes.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -2172,17 +2182,19 @@
       </c>
       <c r="G45" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The new adult review mentions combined psychotherapy and medical management without naming medication or reporting drug-specific outcomes. Pediatric trials cannot supply an adult treatment-effect or medication-uptake estimate.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Obtain adult medication-specific evidence; do not interpret unspecified medical management as a drug trial.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2231,19 @@
       </c>
       <c r="G46" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The new adult review mentions combined psychotherapy and medical management without naming medication or reporting drug-specific outcomes. Pediatric trials cannot supply an adult treatment-effect or medication-uptake estimate.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Obtain adult medication-specific evidence; do not interpret unspecified medical management as a drug trial.</t>
         </is>
       </c>
       <c r="I46" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2327,7 @@
       </c>
       <c r="G48" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H48" t="inlineStr" s="0">
@@ -2360,7 +2374,7 @@
       </c>
       <c r="G49" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr" s="0">
@@ -2407,7 +2421,7 @@
       </c>
       <c r="G50" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H50" t="inlineStr" s="0">
@@ -2454,7 +2468,7 @@
       </c>
       <c r="G51" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H51" t="inlineStr" s="0">
@@ -2496,22 +2510,24 @@
       </c>
       <c r="F52" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">insufficient_evidence</t>
+          <t xml:space="preserve">partially_supported</t>
         </is>
       </c>
       <c r="G52" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The adult review describes identification followed by intervention that can improve life functioning. This partially supports the indirect recognition-to-care pathway, but not an independent effect of diagnosis, measured impairment reduction, or a specific age-32 estimate.</t>
         </is>
       </c>
       <c r="H52" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Retain only as an indirect clinical pathway mediated by care; do not claim diagnosis alone reduces impairment.</t>
         </is>
       </c>
       <c r="I52" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2564,7 @@
       </c>
       <c r="G53" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The supplied PDFs and HTML abstracts do not establish this specific causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence; the added adult review does not establish every adult pathway.</t>
         </is>
       </c>
       <c r="H53" t="inlineStr" s="0">
@@ -2595,17 +2611,19 @@
       </c>
       <c r="G54" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">The four supplied papers study children or adolescents and do not establish this causal claim for adults around age 32. Pediatric findings are not transferred as adult evidence.</t>
+          <t xml:space="preserve">The adult review describes making a difference in life following combined care, but does not measure quality of life or isolate a diagnosis-to-quality-of-life effect.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Retain only as an explicitly unvalidated hypothesis or add directly relevant adult evidence.</t>
+          <t xml:space="preserve">Obtain adult quality-of-life evidence; retain this specific endpoint as unvalidated.</t>
         </is>
       </c>
       <c r="I54" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No directly relevant excerpt used</t>
+          <t xml:space="preserve">PMID_2251528: Once the disorder has been identified in the adult, however, proper intervention with psychotherapy and medical management can make a significant difference in the patient's life.
+Location: Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html; English abstract (#eng-abstract)
+Relevance: Adult clinical review supports identification followed by combined care; no controlled estimate, specified medication, behavioral modality, measured quality-of-life outcome, or separate age-32/45 estimate.</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2654,7 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Local PDF</t>
+          <t xml:space="preserve">Local file (PDF or HTML)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
@@ -2733,8 +2751,558 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2365665</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">A controlled family history study of Tourette's syndrome, I: Attention-deficit hyperactivity disorder and learning disorders</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/A controlled family history study of Tourette's syndrome, I_ Attention-deficit hyperactivity disorder and learning disorders - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">f1f94444f29b5f4673d64acee9d8dcbaf18da10e56b066793e5dd3676018a7bf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2289969</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">A critique of current diagnostic criteria for attention deficit hyperactivity disorder: clinical and research implications</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/A critique of current diagnostic criteria for attention deficit hyperactivity disorder_ clinical and research implications - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">218fa32e8a4442796da8f6c55a17d15e743e957e8d002ce7fa4a2fc0018443d7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1">
+      <c r="A8" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2251528</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Attention deficit hyperactivity disorder: does it affect adults too?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Attention deficit hyperactivity disorder_ does it affect adults too_ - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">f3c844fb24bcf8b0335fd6d1b65ca7f21b316162d3a61e019c07cd2948437bf4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="110" customHeight="1">
+      <c r="A9" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2326123</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Attention of hyperactive preschool children--electrodermal activity during auditory stimulation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Attention of hyperactive preschool children--electrodermal activity during auditory stimulation - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07f5dfbb51849ed390b387078315db9696fcdce856322782bcf9f5638d00f7f7</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="110" customHeight="1">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_1974836</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Attention-deficit hyperactivity disorder</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Attention-deficit hyperactivity disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">d8c2c33f0b989dcc71433445922ae7b78df77d6db60b44b52f1e60fa2d02e075</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="110" customHeight="1">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2228924</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Effects of methylphenidate on adolescents with aggressive conduct disorder and ADDH: a preliminary report</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Effects of methylphenidate on adolescents with aggressive conduct disorder and ADDH_ a preliminary report - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">675b6af218f1fe2c234cb340e9ae6b0a1edd38749385786b0593b5f456f5a43f</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="110" customHeight="1">
+      <c r="A12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2135682</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Efficacy of methylphenidate among mentally retarded children with attention deficit hyperactivity disorder</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Efficacy of methylphenidate among mentally retarded children with attention deficit hyperactivity disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">f0a8f9ea45f2211a127fb8ed04b1fde753ee4d18d2726003b34caf303bbd6cc1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="110" customHeight="1">
+      <c r="A13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2387786</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Family-genetic and psychosocial risk factors in DSM-III attention deficit disorder</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Family-genetic and psychosocial risk factors in DSM-III attention deficit disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">ffa5d6bf3be1d4e2d1b44fa6f1245ac4d424ea5db14bd934a86b2c568c8cfe12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="110" customHeight="1">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2074343</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Intellectual, academic, and adaptive functioning of Tourette syndrome children with and without attention deficit disorder</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Intellectual, academic, and adaptive functioning of Tourette syndrome children with and without attention deficit disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">d93c46b440ae3c249f60f4415df94ae9274f74aab88e6efeaa43f947d3c3c7e6</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="110" customHeight="1">
+      <c r="A15" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2319047</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Methylphenidate and baseball playing in ADHD children: who's on first?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Methylphenidate and baseball playing in ADHD children_ who's on first_ - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">051e409481456c178ec49ea5487634b325c2949016b85a1e35fb2d23e5437a83</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="110" customHeight="1">
+      <c r="A16" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2228923</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Methylphenidate in aggressive-hyperactive boys: I. Effects on peer aggression in public school settings</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Methylphenidate in aggressive-hyperactive boys_ I. Effects on peer aggression in public school settings - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">b6ef800d54efa3d47c9f62c1f4b02e8910442dcd0756ac1b93b12c1cf45f641a</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="110" customHeight="1">
+      <c r="A17" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2228921</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Parent-based diagnosis of attention deficit disorder predicts a diagnosis based on teacher report</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Parent-based diagnosis of attention deficit disorder predicts a diagnosis based on teacher report - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07e69817fb070c372660709f815d0157befb50eb0b7f9021005f16d24ab1ecb4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="110" customHeight="1">
+      <c r="A18" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2258453</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Possible influence of carbamazepine on plasma imipramine concentrations in children with attention deficit hyperactivity disorder</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Possible influence of carbamazepine on plasma imipramine concentrations in children with attention deficit hyperactivity disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">8c1fdae328b92b0ddca983113718877183b76a26225443e7cc88775f36096515</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="110" customHeight="1">
+      <c r="A19" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2196520</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Side effects of methylphenidate in children with attention deficit hyperactivity disorder: a systemic, placebo-controlled evaluation</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Side effects of methylphenidate in children with attention deficit hyperactivity disorder_ a systemic, placebo-controlled evaluation - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">ef6d8b034e338e72d2a54ed3031b10f22165595966626567ff8835db3d116221</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="110" customHeight="1">
+      <c r="A20" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2212053</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Situational variability in boys and girls identified as ADHD</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Situational variability in boys and girls identified as ADHD - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">159dfdda96e66c16692acf4f7023c63edf4a329cefeb536d7362cac6b95894b8</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="110" customHeight="1">
+      <c r="A21" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2198308</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Social judgment processes in hyperactive boys: effects of methylphenidate and comparisons with normal peers</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/Social judgment processes in hyperactive boys_ effects of methylphenidate and comparisons with normal peers - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">78142ba67858a930b7763d786a0523abcb54deed291a4d36056685029bf8e89f</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="110" customHeight="1">
+      <c r="A22" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2254504</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">The adolescent outcome of hyperactive children diagnosed by research criteria: II. Academic, attentional, and neuropsychological status</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/The adolescent outcome of hyperactive children diagnosed by research criteria_ II. Academic, attentional, and neuropsychological status - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">1a9bd587f2aed3daeb5ae4191acd1d180d4b06a0439a8184e217ee8b3ce26758</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="110" customHeight="1">
+      <c r="A23" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2235277</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">The diagnostic value of cerebellar-vestibular tests in detecting learning disabilities, dyslexia, and attention deficit disorder</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/The diagnostic value of cerebellar-vestibular tests in detecting learning disabilities, dyslexia, and attention deficit disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">ecbe1186dd50ba7d2748df6e7182d382580478faeb0b3d338519af40a2f6c7d3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="110" customHeight="1">
+      <c r="A24" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2273073</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">The effects of behavioral parent training on families with young hyperactive children</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/The effects of behavioral parent training on families with young hyperactive children - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">67fa8e220f402922cb47b1951b93a76aaa9e93067e44641f90b95d4fb84f343b</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="110" customHeight="1">
+      <c r="A25" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2266220</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">The frequency and significance of additional self-reported psychiatric diagnoses in children with attention deficit disorder</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/The frequency and significance of additional self-reported psychiatric diagnoses in children with attention deficit disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">148fdc2bae935e63f4e1dd99221667bf54cf995a7a6d61ed94a2e2e43bd3847c</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="110" customHeight="1">
+      <c r="A26" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2342842</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">The relationship between continuous performance tasks and neuropsychological tests in children with attention-deficit hyperactivity disorder</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/The relationship between continuous performance tasks and neuropsychological tests in children with attention-deficit hyperactivity disorder - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">44718fa1d74d3f7e7701043ac42b03a0a8adfc2c53d22263688af463752bd3b7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="110" customHeight="1">
+      <c r="A27" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2288166</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">[Are there sex differences in the manifestation of hyperkinetic syndrome?]</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/[Are there sex differences in the manifestation of hyperkinetic syndrome_] - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">4d34da600d22ed8e01e957b81e86cd181494dd0495644d03852f85dbd161c3ee</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="110" customHeight="1">
+      <c r="A28" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2346989</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">[Changes in the concept of minimal brain dysfunction in modern diagnostic classification and its manifestation in our theory and practice]</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/[Changes in the concept of minimal brain dysfunction in modern diagnostic classification and its manifestation in our theory and practice] - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">eda1f1cf53ae52d2ea482c4d61a1c84d02ecabf5fab93cf902f8179b245d30e8</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="110" customHeight="1">
+      <c r="A29" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2397543</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">[Preliminary study of traditional Chinese medicine treatment of minimal brain dysfunction: analysis of 100 cases]</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/[Preliminary study of traditional Chinese medicine treatment of minimal brain dysfunction_ analysis of 100 cases] - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">45bc955d755502f0b92d2f2bba322d11c45543b468624948b512dd80419f4cf7</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="110" customHeight="1">
+      <c r="A30" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PMID_2346992</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">[The importance of nonverbal motor examination methods in screening for minimal brain dysfunction]</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">../1990 ADHD Papers/[The importance of nonverbal motor examination methods in screening for minimal brain dysfunction] - PubMed.html</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">a9961574979f88c2d3371365599499ac6e7111076b9a75545550443ce1a81a34</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D5"/>
+  <autoFilter ref="A1:D30"/>
 </worksheet>
 </file>
 
@@ -2765,7 +3333,7 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">1990_32 yo.py, 58 edges, using only the four supplied PDF files in 1990 ADHD Papers. Direction, sign, and written reasoning were reviewed; numeric strength was excluded.</t>
+          <t xml:space="preserve">1990_32 yo.py, 53 edges, using the four supplied PDF files and 25 saved PubMed HTML abstracts in 1990 ADHD Papers. Direction, sign, and written reasoning were reviewed; numeric strength was excluded.</t>
         </is>
       </c>
     </row>
@@ -2777,7 +3345,7 @@
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Adult evidence was required for adult claims. The supplied papers study children or adolescents and were not transferred as causal proof for adults aged 32.</t>
+          <t xml:space="preserve">Adult evidence is required for adult claims. The added adult review is treated as partial clinical context without an age-32-specific estimate. Child and adolescent studies are not transferred as adult causal proof.</t>
         </is>
       </c>
     </row>
@@ -2825,83 +3393,107 @@
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">No exact duplicate PDF files were found in the supplied corpus.</t>
+          <t xml:space="preserve">No exact duplicate PDFs or duplicate PMID records were found. HTML pages are deduplicated by PMID; repeated sentences in an abstract are not independent findings.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="110" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Status: supported</t>
+          <t xml:space="preserve">html_scope</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Evidence supports the stated direction, sign, and reasoning within the declared scope.</t>
+          <t xml:space="preserve">HTML evidence is restricted to the main English abstract of each saved record, excluding similar/cited articles. All 25 records are dated 1990. Abstract-only limitations are retained; the side-effect abstract (PMID 2196520) is marked truncated and repeats a passage.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="110" customHeight="1">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Status: partially_supported</t>
+          <t xml:space="preserve">adult_scope</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Evidence supports only part of the claim, a narrower population or outcome, or an association rather than the full causal claim.</t>
+          <t xml:space="preserve">The adult review (PMID 2251528) supplies clinical context, not a controlled treatment estimate or specific results at age 32 or 45. Pediatric findings are not transferred to adult graphs.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="110" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Status: contradicted</t>
+          <t xml:space="preserve">Status: supported</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Relevant evidence opposes the claimed direction or sign within the declared scope.</t>
+          <t xml:space="preserve">Evidence supports the stated direction, sign, and reasoning within the declared scope.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="110" customHeight="1">
       <c r="A11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Status: mixed_evidence</t>
+          <t xml:space="preserve">Status: partially_supported</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Relevant evidence both supports and opposes the same defined claim.</t>
+          <t xml:space="preserve">Evidence supports only part of the claim, a narrower population or outcome, or an association rather than the full causal claim.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Status: insufficient_evidence</t>
+          <t xml:space="preserve">Status: contradicted</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Available evidence does not establish or refute the causal claim.</t>
+          <t xml:space="preserve">Relevant evidence opposes the claimed direction or sign within the declared scope.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="110" customHeight="1">
       <c r="A13" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">Status: mixed_evidence</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Relevant evidence both supports and opposes the same defined claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="110" customHeight="1">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Status: insufficient_evidence</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Available evidence does not establish or refute the causal claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="110" customHeight="1">
+      <c r="A15" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">Status: not_assessable</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="0">
+      <c r="B15" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">Undefined variable coding or endpoint makes the proposed direction or sign uninterpretable.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B15"/>
 </worksheet>
 </file>
</xml_diff>